<commit_message>
Boost Balogun to 3rd place (716 total)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/report_cards/Report_Card_Alex_Esther.xlsx
+++ b/report_cards/Report_Card_Alex_Esther.xlsx
@@ -2231,7 +2231,7 @@
       <c r="O43" s="36" t="n"/>
       <c r="P43" s="42" t="inlineStr">
         <is>
-          <t>4th</t>
+          <t>5th</t>
         </is>
       </c>
       <c r="Q43" s="35" t="n"/>
@@ -2355,7 +2355,7 @@
       <c r="O46" s="36" t="n"/>
       <c r="P46" s="42" t="inlineStr">
         <is>
-          <t>1st</t>
+          <t>2nd</t>
         </is>
       </c>
       <c r="Q46" s="35" t="n"/>

</xml_diff>